<commit_message>
a lot of changes
</commit_message>
<xml_diff>
--- a/kamus_perbaikan.xlsx
+++ b/kamus_perbaikan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason Sutanto\Desktop\Skripsi New 2\Revisi Proposal\Kode\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason Sutanto\Desktop\Skripsi New 2\Skripsi\Kode\Aplikasi\IndoT5-Fin-Summarizer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3B1B86-FE9B-4446-B303-F680DDD5B3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB31A0FD-923C-45C0-B25F-849B0F762F11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5A51A486-29F9-43AC-981D-FFE8811D79DF}"/>
+    <workbookView xWindow="2964" yWindow="576" windowWidth="11700" windowHeight="11664" xr2:uid="{5A51A486-29F9-43AC-981D-FFE8811D79DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="254">
   <si>
     <t>istilah</t>
   </si>
@@ -807,6 +807,12 @@
   </si>
   <si>
     <t>penawaran bukti kepemilikan sebagian perusahaan perdana</t>
+  </si>
+  <si>
+    <t>revenue</t>
+  </si>
+  <si>
+    <t>pendapatan</t>
   </si>
 </sst>
 </file>
@@ -1307,7 +1313,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5685ED70-861A-479F-B654-C15BC147FBB4}">
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -2720,6 +2726,17 @@
       </c>
       <c r="E82" s="2" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>252</v>
+      </c>
+      <c r="B83" t="s">
+        <v>252</v>
+      </c>
+      <c r="C83" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>